<commit_message>
updated Testcase withcreate Account
</commit_message>
<xml_diff>
--- a/src/test/resources/Testdata/data.xlsx
+++ b/src/test/resources/Testdata/data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D95B2B24-E426-4029-94D1-DA2A181E2BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{0074F3BE-0EE9-4ABE-8D49-1E6B811B1E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{10CD009A-6023-4229-BBF5-797C429F342B}"/>
   </bookViews>
@@ -18,21 +18,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
   <si>
     <t>username</t>
   </si>
@@ -158,6 +149,12 @@
   </si>
   <si>
     <t>admin135</t>
+  </si>
+  <si>
+    <t>mngr666481</t>
+  </si>
+  <si>
+    <t>nudurYm</t>
   </si>
 </sst>
 </file>
@@ -554,8 +551,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58A41266-E193-43DE-B354-7BADC994ADAE}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -675,6 +675,14 @@
       </c>
       <c r="B15" s="2" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>